<commit_message>
feat: Scrape EVE Online Ore Prices
Co-authored-by: traeagent <traeagent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/EVE_Standard_Ore_Prices.xlsx
+++ b/EVE_Standard_Ore_Prices.xlsx
@@ -581,10 +581,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="26" customHeight="1">
+    <row r="3" ht="40" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Pricing: average of ALL orders on each item page, IQR 1.5x outliers removed; BUY and SELL computed separately. Grade IV, Compressed, Batch Compressed excluded. N/A = no matching orders.</t>
+          <t>Pricing: for each ore, BEST SELL = lowest sell order, BEST BUY = highest buy order. Only orders within 1.5x of the corresponding BEST value are averaged (SELL: [BEST SELL, BEST SELL x1.5]; BUY: [BEST BUY / 1.5, BEST BUY]); orders deviating beyond 1.5x are excluded. BUY and SELL computed separately. Grade IV, Compressed and Batch Compressed excluded. N/A = no orders in range.</t>
         </is>
       </c>
     </row>
@@ -596,12 +596,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Acc SELL Price</t>
+          <t>Avg SELL Price</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Acc BUY Price</t>
+          <t>Avg BUY Price</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>5472.29</v>
+        <v>5633.09</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>2127.57</v>
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="C8" s="11" t="n">
-        <v>3018</v>
+        <v>3526.33</v>
       </c>
     </row>
     <row r="9">
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>2661.67</v>
+        <v>3580</v>
       </c>
     </row>
     <row r="11">
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>10731.11</v>
+        <v>11158</v>
       </c>
       <c r="C12" s="8" t="n">
         <v>6021.67</v>
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="C13" s="11" t="n">
-        <v>3255</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="14">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>6570</v>
+        <v>8140</v>
       </c>
     </row>
     <row r="16">
@@ -725,10 +725,10 @@
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>41050</v>
+        <v>2416.67</v>
       </c>
       <c r="C17" s="8" t="n">
-        <v>1944.33</v>
+        <v>1880.86</v>
       </c>
     </row>
     <row r="18">
@@ -741,7 +741,7 @@
         <v>3605.5</v>
       </c>
       <c r="C18" s="11" t="n">
-        <v>1527</v>
+        <v>2303.5</v>
       </c>
     </row>
     <row r="19">
@@ -778,7 +778,7 @@
         <v>4665</v>
       </c>
       <c r="C22" s="8" t="n">
-        <v>2826.66</v>
+        <v>4426.2</v>
       </c>
     </row>
     <row r="23">
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>2925.67</v>
+        <v>4388</v>
       </c>
     </row>
     <row r="24">
@@ -841,7 +841,7 @@
         <v>4004.5</v>
       </c>
       <c r="C28" s="11" t="n">
-        <v>2637.5</v>
+        <v>2682</v>
       </c>
     </row>
     <row r="29">
@@ -927,10 +927,10 @@
         </is>
       </c>
       <c r="B37" s="8" t="n">
-        <v>4961.17</v>
+        <v>4907.12</v>
       </c>
       <c r="C37" s="8" t="n">
-        <v>820</v>
+        <v>1229.5</v>
       </c>
     </row>
     <row r="38">
@@ -984,7 +984,7 @@
         </is>
       </c>
       <c r="C42" s="8" t="n">
-        <v>54.33</v>
+        <v>161</v>
       </c>
     </row>
     <row r="43">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="B47" s="8" t="n">
-        <v>288.82</v>
+        <v>217.63</v>
       </c>
       <c r="C47" s="8" t="n">
         <v>41.5</v>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="B52" s="8" t="n">
-        <v>373.47</v>
+        <v>247.18</v>
       </c>
       <c r="C52" s="8" t="n">
-        <v>26.08</v>
+        <v>151.8</v>
       </c>
     </row>
     <row r="53">
@@ -1154,7 +1154,7 @@
         </is>
       </c>
       <c r="C57" s="8" t="n">
-        <v>60.71</v>
+        <v>135</v>
       </c>
     </row>
     <row r="58">
@@ -1207,10 +1207,10 @@
         </is>
       </c>
       <c r="B62" s="8" t="n">
-        <v>2346.67</v>
+        <v>2335</v>
       </c>
       <c r="C62" s="8" t="n">
-        <v>1402.6</v>
+        <v>1477.17</v>
       </c>
     </row>
     <row r="63">
@@ -1240,7 +1240,7 @@
         </is>
       </c>
       <c r="C64" s="8" t="n">
-        <v>1150</v>
+        <v>1724.5</v>
       </c>
     </row>
     <row r="66">
@@ -1264,7 +1264,7 @@
         </is>
       </c>
       <c r="C67" s="8" t="n">
-        <v>81.29000000000001</v>
+        <v>81.28</v>
       </c>
     </row>
     <row r="68">
@@ -1313,7 +1313,7 @@
         </is>
       </c>
       <c r="B72" s="8" t="n">
-        <v>3643</v>
+        <v>999.95</v>
       </c>
       <c r="C72" s="8" t="n">
         <v>506.45</v>
@@ -1331,7 +1331,7 @@
         </is>
       </c>
       <c r="C73" s="11" t="n">
-        <v>530.03</v>
+        <v>530.02</v>
       </c>
     </row>
     <row r="74">
@@ -1344,7 +1344,7 @@
         <v>1339.5</v>
       </c>
       <c r="C74" s="8" t="n">
-        <v>556.67</v>
+        <v>570</v>
       </c>
     </row>
     <row r="76">
@@ -1363,10 +1363,10 @@
         </is>
       </c>
       <c r="B77" s="8" t="n">
-        <v>1281.06</v>
+        <v>1160.58</v>
       </c>
       <c r="C77" s="8" t="n">
-        <v>916.04</v>
+        <v>923.16</v>
       </c>
     </row>
     <row r="78">
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="C82" s="8" t="n">
-        <v>335.17</v>
+        <v>502.75</v>
       </c>
     </row>
     <row r="83">
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="C83" s="11" t="n">
-        <v>392.9</v>
+        <v>589.35</v>
       </c>
     </row>
     <row r="84">
@@ -1448,7 +1448,7 @@
         </is>
       </c>
       <c r="C84" s="8" t="n">
-        <v>343.04</v>
+        <v>514.55</v>
       </c>
     </row>
     <row r="86">
@@ -1467,7 +1467,7 @@
         </is>
       </c>
       <c r="B87" s="8" t="n">
-        <v>2303.99</v>
+        <v>451.6</v>
       </c>
       <c r="C87" s="8" t="n">
         <v>233.34</v>
@@ -1515,10 +1515,10 @@
         </is>
       </c>
       <c r="B92" s="8" t="n">
-        <v>819.89</v>
+        <v>623.47</v>
       </c>
       <c r="C92" s="8" t="n">
-        <v>449.25</v>
+        <v>481.58</v>
       </c>
     </row>
     <row r="93">
@@ -1528,7 +1528,7 @@
         </is>
       </c>
       <c r="B93" s="11" t="n">
-        <v>387.37</v>
+        <v>158.95</v>
       </c>
       <c r="C93" s="11" t="n">
         <v>145.81</v>
@@ -1541,7 +1541,7 @@
         </is>
       </c>
       <c r="B94" s="8" t="n">
-        <v>379.01</v>
+        <v>169</v>
       </c>
       <c r="C94" s="8" t="n">
         <v>144.57</v>
@@ -1644,7 +1644,7 @@
         <v>18995</v>
       </c>
       <c r="C104" s="8" t="n">
-        <v>10703.67</v>
+        <v>16055</v>
       </c>
     </row>
     <row r="106">
@@ -1666,7 +1666,7 @@
         <v>30</v>
       </c>
       <c r="C107" s="8" t="n">
-        <v>9.33</v>
+        <v>17.01</v>
       </c>
     </row>
     <row r="108">
@@ -1689,10 +1689,10 @@
         </is>
       </c>
       <c r="B109" s="8" t="n">
-        <v>41.7</v>
+        <v>17.53</v>
       </c>
       <c r="C109" s="8" t="n">
-        <v>11.35</v>
+        <v>11.01</v>
       </c>
     </row>
     <row r="111">
@@ -1716,7 +1716,7 @@
         </is>
       </c>
       <c r="C112" s="8" t="n">
-        <v>300.64</v>
+        <v>450.95</v>
       </c>
     </row>
     <row r="113">
@@ -1731,7 +1731,7 @@
         </is>
       </c>
       <c r="C113" s="11" t="n">
-        <v>302.64</v>
+        <v>453.95</v>
       </c>
     </row>
     <row r="114">
@@ -1765,10 +1765,10 @@
         </is>
       </c>
       <c r="B117" s="8" t="n">
-        <v>384.16</v>
+        <v>121.7</v>
       </c>
       <c r="C117" s="8" t="n">
-        <v>36.46</v>
+        <v>97.03</v>
       </c>
     </row>
     <row r="118">
@@ -1778,7 +1778,7 @@
         </is>
       </c>
       <c r="B118" s="11" t="n">
-        <v>128</v>
+        <v>124.18</v>
       </c>
       <c r="C118" s="11" t="n">
         <v>82.26000000000001</v>
@@ -1791,7 +1791,7 @@
         </is>
       </c>
       <c r="B119" s="8" t="n">
-        <v>133.66</v>
+        <v>120.07</v>
       </c>
       <c r="C119" s="8" t="n">
         <v>85.27</v>
@@ -1813,7 +1813,7 @@
         </is>
       </c>
       <c r="B122" s="8" t="n">
-        <v>49.13</v>
+        <v>33.84</v>
       </c>
       <c r="C122" s="8" t="n">
         <v>27.16</v>
@@ -1826,10 +1826,10 @@
         </is>
       </c>
       <c r="B123" s="11" t="n">
-        <v>40.36</v>
+        <v>39.41</v>
       </c>
       <c r="C123" s="11" t="n">
-        <v>26.94</v>
+        <v>27.63</v>
       </c>
     </row>
     <row r="124">
@@ -1839,10 +1839,10 @@
         </is>
       </c>
       <c r="B124" s="8" t="n">
-        <v>57.23</v>
+        <v>35.8</v>
       </c>
       <c r="C124" s="8" t="n">
-        <v>28.06</v>
+        <v>29.15</v>
       </c>
     </row>
     <row r="126">
@@ -1864,7 +1864,7 @@
         <v>45153.33</v>
       </c>
       <c r="C127" s="8" t="n">
-        <v>9.17</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="128">
@@ -1917,10 +1917,10 @@
         </is>
       </c>
       <c r="B132" s="8" t="n">
-        <v>54.24</v>
+        <v>28.55</v>
       </c>
       <c r="C132" s="8" t="n">
-        <v>16.79</v>
+        <v>22.02</v>
       </c>
     </row>
     <row r="133">
@@ -1930,10 +1930,10 @@
         </is>
       </c>
       <c r="B133" s="11" t="n">
-        <v>25.99</v>
+        <v>25.98</v>
       </c>
       <c r="C133" s="11" t="n">
-        <v>16.06</v>
+        <v>21.58</v>
       </c>
     </row>
     <row r="134">
@@ -1943,10 +1943,10 @@
         </is>
       </c>
       <c r="B134" s="8" t="n">
-        <v>73.06999999999999</v>
+        <v>32.92</v>
       </c>
       <c r="C134" s="8" t="n">
-        <v>19.15</v>
+        <v>22.56</v>
       </c>
     </row>
     <row r="136">
@@ -1965,10 +1965,10 @@
         </is>
       </c>
       <c r="B137" s="8" t="n">
-        <v>14000</v>
+        <v>10000</v>
       </c>
       <c r="C137" s="8" t="n">
-        <v>2500.01</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="138">
@@ -1983,7 +1983,7 @@
         </is>
       </c>
       <c r="C138" s="11" t="n">
-        <v>2500.01</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="139">
@@ -1998,7 +1998,7 @@
         </is>
       </c>
       <c r="C139" s="8" t="n">
-        <v>2750.01</v>
+        <v>5500</v>
       </c>
     </row>
     <row r="141">
@@ -2017,7 +2017,7 @@
         </is>
       </c>
       <c r="B142" s="8" t="n">
-        <v>57.67</v>
+        <v>21.54</v>
       </c>
       <c r="C142" s="8" t="n">
         <v>14.78</v>
@@ -2030,7 +2030,7 @@
         </is>
       </c>
       <c r="B143" s="11" t="n">
-        <v>23.37</v>
+        <v>21.71</v>
       </c>
       <c r="C143" s="11" t="n">
         <v>16.72</v>
@@ -2043,7 +2043,7 @@
         </is>
       </c>
       <c r="B144" s="8" t="n">
-        <v>24.03</v>
+        <v>23.69</v>
       </c>
       <c r="C144" s="8" t="n">
         <v>15.94</v>
@@ -2065,10 +2065,10 @@
         </is>
       </c>
       <c r="B147" s="8" t="n">
-        <v>16577.5</v>
+        <v>15802.86</v>
       </c>
       <c r="C147" s="8" t="n">
-        <v>5311.75</v>
+        <v>7967</v>
       </c>
     </row>
     <row r="148">
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="B152" s="8" t="n">
-        <v>13824.44</v>
+        <v>13430</v>
       </c>
       <c r="C152" s="8" t="n">
         <v>4759</v>
@@ -2133,7 +2133,7 @@
         <v>15000</v>
       </c>
       <c r="C153" s="11" t="n">
-        <v>3426.67</v>
+        <v>5140</v>
       </c>
     </row>
     <row r="154">
@@ -2148,7 +2148,7 @@
         </is>
       </c>
       <c r="C154" s="8" t="n">
-        <v>3370.34</v>
+        <v>5055.5</v>
       </c>
     </row>
     <row r="156">
@@ -2167,7 +2167,7 @@
         </is>
       </c>
       <c r="B157" s="8" t="n">
-        <v>320</v>
+        <v>200</v>
       </c>
       <c r="C157" s="8" t="n">
         <v>4.51</v>
@@ -2226,7 +2226,7 @@
         <v>4500</v>
       </c>
       <c r="C162" s="8" t="n">
-        <v>335.5</v>
+        <v>503.25</v>
       </c>
     </row>
     <row r="163">
@@ -2254,7 +2254,7 @@
         </is>
       </c>
       <c r="C164" s="8" t="n">
-        <v>368.04</v>
+        <v>552.05</v>
       </c>
     </row>
     <row r="166">
@@ -2273,7 +2273,7 @@
         </is>
       </c>
       <c r="B167" s="8" t="n">
-        <v>137.72</v>
+        <v>14.51</v>
       </c>
       <c r="C167" s="8" t="n">
         <v>10.14</v>
@@ -2286,7 +2286,7 @@
         </is>
       </c>
       <c r="B168" s="11" t="n">
-        <v>14.87</v>
+        <v>12.99</v>
       </c>
       <c r="C168" s="11" t="n">
         <v>10.65</v>
@@ -2299,7 +2299,7 @@
         </is>
       </c>
       <c r="B169" s="8" t="n">
-        <v>13.65</v>
+        <v>13.53</v>
       </c>
       <c r="C169" s="8" t="n">
         <v>10.44</v>
@@ -2321,7 +2321,7 @@
         </is>
       </c>
       <c r="B172" s="8" t="n">
-        <v>349.92</v>
+        <v>331.17</v>
       </c>
       <c r="C172" s="8" t="n">
         <v>249.78</v>
@@ -2339,7 +2339,7 @@
         </is>
       </c>
       <c r="C173" s="11" t="n">
-        <v>5536.67</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="174">
@@ -2354,7 +2354,7 @@
         </is>
       </c>
       <c r="C174" s="8" t="n">
-        <v>5603.33</v>
+        <v>10000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>